<commit_message>
feat(ner): benchmark 5-fold OOF fine-tuning IndoBERT-ner-gold (NER-ENCODER-002)
- Daftarkan treamyracle/indobert-ner-gold ke tests/benchmark_ner_encoders.py dengan konfigurasi setara mDeBERTa & XLM-RoBERTa
- Eksekusi 5-fold stratified cross-validation OOF training: IndoBERT meraih 44.52% framework exact (+31.72pt vs pre-trained)
- Nama kegiatan exact melonjak ke 43.24% (fuzzy 78.38%), mengungguli DeBERTa (25.68%) dan XLM-RoBERTa (35.14%)
- Catat metrik resmi di docs/experiments_ledger.md dan docs/report/runs_summary.md
- Perbarui skrip generator dan workbook docs/report/komparasi_ner_encoder_dan_pipeline.xlsx pada seluruh 4 sheet evaluasi
</commit_message>
<xml_diff>
--- a/docs/report/komparasi_ner_encoder_dan_pipeline.xlsx
+++ b/docs/report/komparasi_ner_encoder_dan_pipeline.xlsx
@@ -213,16 +213,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -250,6 +250,15 @@
     <xf numFmtId="168" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -257,15 +266,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -984,275 +984,305 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>5-Fold CV Token Classif.</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.4452</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>[38.59%, 50.82%]</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.4324</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.5769</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0.3649</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0.4909</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>700.1 detik (~11.7m)</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>4.65 GB</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>BEST ENCODER (PASS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Direct Gemini 3.1 Flash Lite</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Two-Stage Tesseract-to-LLM</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.6324</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D10" s="16" t="n">
         <v>0.7378</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>[58.78%, 68.92%]</t>
         </is>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.6216</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.5946</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H10" s="18" t="n">
         <v>0.5946</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I10" s="18" t="n">
         <v>0.6757</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J10" s="18" t="n">
         <v>0.6757</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K10" s="18" t="n">
         <v>0.6622</v>
       </c>
-      <c r="L9" s="17" t="inlineStr">
+      <c r="L10" s="17" t="inlineStr">
         <is>
           <t>100.6 detik (1.36s/c)</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr">
+      <c r="M10" s="17" t="inlineStr">
         <is>
           <t>Rp703 (~Rp9.50/c)</t>
         </is>
       </c>
-      <c r="N9" s="15" t="inlineStr">
+      <c r="N10" s="15" t="inlineStr">
         <is>
           <t>PRODUKSI AKTIF (Opt A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Composite v4.x (Pure OCR)</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Pure 100% Tesseract OCR + Rules</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>0.771</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>0.8516</v>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>[72.10%, 81.80%]</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>0.8947000000000001</v>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="J10" s="13" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="K10" s="13" t="n">
-        <v>0.6847</v>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
-        <is>
-          <t>0 detik (Offline)</t>
-        </is>
-      </c>
-      <c r="M10" s="12" t="inlineStr">
-        <is>
-          <t>0 GB (CPU Local)</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr">
-        <is>
-          <t>Baseline Pure OCR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Composite v4.x (Pure OCR)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Pure 100% Tesseract OCR + Rules</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.8516</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>[72.10%, 81.80%]</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.8947000000000001</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>0.6847</v>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>0 detik (Offline)</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>0 GB (CPU Local)</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Baseline Pure OCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>Combined v4.2 (Hybrid)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Hybrid Layer + 3 Pillars &amp; Crop</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C12" s="11" t="n">
         <v>0.8742</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D12" s="11" t="n">
         <v>0.9</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>[83.50%, 91.20%]</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F12" s="13" t="n">
         <v>0.797</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G12" s="13" t="n">
         <v>0.923</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H12" s="13" t="n">
         <v>0.662</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I12" s="13" t="n">
         <v>0.909</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J12" s="13" t="n">
         <v>0.909</v>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="K12" s="13" t="n">
         <v>0.7682</v>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L12" s="12" t="inlineStr">
         <is>
           <t>0 detik (Offline)</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M12" s="12" t="inlineStr">
         <is>
           <t>0 GB (CPU Local)</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="N12" s="10" t="inlineStr">
         <is>
           <t>Fallback Produksi</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Rata-rata Model Teruji</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Rata-rata Metrik</t>
         </is>
       </c>
-      <c r="C12" s="21">
-        <f>AVERAGE(C5:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="21">
-        <f>AVERAGE(D5:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="22" t="inlineStr"/>
-      <c r="F12" s="22" t="inlineStr"/>
-      <c r="G12" s="22" t="inlineStr"/>
-      <c r="H12" s="22" t="inlineStr"/>
-      <c r="I12" s="22" t="inlineStr"/>
-      <c r="J12" s="22" t="inlineStr"/>
-      <c r="K12" s="22" t="inlineStr"/>
-      <c r="L12" s="22" t="inlineStr"/>
-      <c r="M12" s="22" t="inlineStr"/>
-      <c r="N12" s="22" t="inlineStr"/>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="C13" s="21">
+        <f>AVERAGE(C5:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="21">
+        <f>AVERAGE(D5:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="22" t="inlineStr"/>
+      <c r="F13" s="22" t="inlineStr"/>
+      <c r="G13" s="22" t="inlineStr"/>
+      <c r="H13" s="22" t="inlineStr"/>
+      <c r="I13" s="22" t="inlineStr"/>
+      <c r="J13" s="22" t="inlineStr"/>
+      <c r="K13" s="22" t="inlineStr"/>
+      <c r="L13" s="22" t="inlineStr"/>
+      <c r="M13" s="22" t="inlineStr"/>
+      <c r="N13" s="22" t="inlineStr"/>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>ANALISIS DELTA PERFORMANSI VS BASELINE PRE-TRAINED NER V1 (INDOBERT)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Model Komparasi</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Baseline Exact</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Model Exact</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Peningkatan Mutlak (pp)</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Peningkatan Relatif (%)</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Kesimpulan Arsitektural</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>IndoBERT Fine-Tuned Gagal (Phase v2)</t>
-        </is>
-      </c>
-      <c r="B16" s="13">
-        <f>C5</f>
-        <v/>
-      </c>
-      <c r="C16" s="13">
-        <f>C6</f>
-        <v/>
-      </c>
-      <c r="D16" s="24">
-        <f>C16-B16</f>
-        <v/>
-      </c>
-      <c r="E16" s="25">
-        <f>(C16-B16)/B16</f>
-        <v/>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Anjlok -11.3pp akibat catastrophic forgetting pada 59 sampel dan ketiadaan weighted loss.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>mDeBERTa-v3-base (86M)</t>
+          <t>IndoBERT Fine-Tuned Gagal (Phase v2)</t>
         </is>
       </c>
       <c r="B17" s="8">
@@ -1260,27 +1290,27 @@
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>C7</f>
-        <v/>
-      </c>
-      <c r="D17" s="26">
+        <f>C6</f>
+        <v/>
+      </c>
+      <c r="D17" s="24">
         <f>C17-B17</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="25">
         <f>(C17-B17)/B17</f>
         <v/>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Peningkatan substansial (+22.04pp) pada recall entitas non-O via FP32 &amp; soft-capping.</t>
+          <t>Anjlok -11.3pp akibat catastrophic forgetting pada 59 sampel dan ketiadaan weighted loss.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>XLM-RoBERTa-large (560M)</t>
+          <t>mDeBERTa-v3-base (86M)</t>
         </is>
       </c>
       <c r="B18" s="13">
@@ -1288,27 +1318,27 @@
         <v/>
       </c>
       <c r="C18" s="13">
-        <f>C8</f>
-        <v/>
-      </c>
-      <c r="D18" s="24">
+        <f>C7</f>
+        <v/>
+      </c>
+      <c r="D18" s="26">
         <f>C18-B18</f>
         <v/>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="27">
         <f>(C18-B18)/B18</f>
         <v/>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Model 560M melompat +30.75pp; representasi BPE multilingual sangat kuat.</t>
+          <t>Peningkatan substansial (+22.04pp) pada recall entitas non-O via FP32 &amp; soft-capping.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Direct Gemini 3.1 Flash Lite</t>
+          <t>XLM-RoBERTa-large (560M)</t>
         </is>
       </c>
       <c r="B19" s="8">
@@ -1316,27 +1346,27 @@
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>C9</f>
-        <v/>
-      </c>
-      <c r="D19" s="26">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="D19" s="24">
         <f>C19-B19</f>
         <v/>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="25">
         <f>(C19-B19)/B19</f>
         <v/>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>LLM murni melampaui seluruh encoder lokal tanpa memerlukan fine-tuning.</t>
+          <t>Model 560M melompat +30.75pp; representasi BPE multilingual sangat kuat.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Composite v4.x (Pure OCR Rules)</t>
+          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
         </is>
       </c>
       <c r="B20" s="13">
@@ -1344,27 +1374,27 @@
         <v/>
       </c>
       <c r="C20" s="13">
-        <f>C10</f>
-        <v/>
-      </c>
-      <c r="D20" s="24">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="D20" s="26">
         <f>C20-B20</f>
         <v/>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="27">
         <f>(C20-B20)/B20</f>
         <v/>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Rule deterministik offline tetap paling unggul pada domain penanggalan &amp; nomor.</t>
+          <t>ENCODER TERBAIK (+31.72pp vs pre-trained, +0.97pp vs XLM-RoBERTa-large, kegiatan melonjak ke 43.2%).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Combined v4.2 (Hybrid Pipeline)</t>
+          <t>Direct Gemini 3.1 Flash Lite</t>
         </is>
       </c>
       <c r="B21" s="8">
@@ -1372,18 +1402,74 @@
         <v/>
       </c>
       <c r="C21" s="8">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="D21" s="24">
+        <f>C21-B21</f>
+        <v/>
+      </c>
+      <c r="E21" s="25">
+        <f>(C21-B21)/B21</f>
+        <v/>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>LLM murni melampaui seluruh encoder lokal tanpa memerlukan fine-tuning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Composite v4.x (Pure OCR Rules)</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C22" s="13">
         <f>C11</f>
         <v/>
       </c>
-      <c r="D21" s="26">
-        <f>C21-B21</f>
-        <v/>
-      </c>
-      <c r="E21" s="27">
-        <f>(C21-B21)/B21</f>
-        <v/>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="D22" s="26">
+        <f>C22-B22</f>
+        <v/>
+      </c>
+      <c r="E22" s="27">
+        <f>(C22-B22)/B22</f>
+        <v/>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Rule deterministik offline tetap paling unggul pada domain penanggalan &amp; nomor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Combined v4.2 (Hybrid Pipeline)</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C23" s="8">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="D23" s="24">
+        <f>C23-B23</f>
+        <v/>
+      </c>
+      <c r="E23" s="25">
+        <f>(C23-B23)/B23</f>
+        <v/>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Pipeline komposit offline terbaik, unggul +74.62pp dibanding baseline NER v1.</t>
         </is>
@@ -1437,15 +1523,20 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>treamyracle/indobert-ner-gold</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>microsoft/mdeberta-v3-base</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>facebookai/xlm-roberta-large</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Rasional &amp; Detail Desain Arsitektural</t>
         </is>
@@ -1459,15 +1550,20 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
+          <t>treamyracle/indobert-ner-gold</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
           <t>microsoft/mdeberta-v3-base</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>facebookai/xlm-roberta-large</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Bobot resmi dari Hugging Face Hub.</t>
         </is>
@@ -1481,17 +1577,22 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
+          <t>334 Juta Parameter</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
           <t>86 Juta Parameter</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>560 Juta Parameter</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>XLM-RoBERTa 6.5x lebih besar dengan kapasitas representasi lebih tinggi.</t>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>IndoBERT-large (334M) di tengah antara mDeBERTa dan XLM-RoBERTa.</t>
         </is>
       </c>
     </row>
@@ -1503,17 +1604,22 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
+          <t>BERT-large (Bidirectional Transformer)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
           <t>DeBERTa-v2 (Disentangled Attention)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>RoBERTa (Transformer Encoder)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>DeBERTa memisahkan representasi isi kata dan posisi relatif.</t>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>IndoBERT fokus monolingual Indonesia vs DeBERTa &amp; XLM-RoBERTa multilingual.</t>
         </is>
       </c>
     </row>
@@ -1525,17 +1631,22 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
+          <t>BertTokenizerFast (Indo4B: 32k)</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
           <t>DeBERTaV2TokenizerFast (SPM: 250k)</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>XLMRobertaTokenizerFast (BPE: 250k)</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>SentencePiece (SPM) vs Byte-Pair Encoding (BPE) multilingual.</t>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Kosakata IndoBERT utuh pada kata Indonesia; tidak terfragmentasi seperti multilingual.</t>
         </is>
       </c>
     </row>
@@ -1555,9 +1666,14 @@
           <t>5-Fold Stratified Cross-Validation</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Stratified berdasarkan distribusi kelengkapan field pada 74 dokumen.</t>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>5-Fold Stratified Cross-Validation</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Identik 100%: stratified berdasarkan kelengkapan field 74 dokumen.</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1693,12 @@
           <t>Weighted Cross Entropy</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Weighted Cross Entropy</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Penyeimbang ketimpangan ekstrem antara kelas O (92%) vs entitas non-O (8%).</t>
         </is>
@@ -1599,7 +1720,12 @@
           <t>Square-Root Inverse-Frequency</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Square-Root Inverse-Frequency</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>w_c = min(sqrt(N_max / N_c), 10.0) mencegah bobot ekstrem meledakkan loss.</t>
         </is>
@@ -1621,9 +1747,14 @@
           <t>10.0x</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Bobot dibatasi maksimal 10.0 (menggantikan bobot 100x yang memicu NaN).</t>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>10.0x</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Bobot dibatasi maksimal 10.0 mencegah divergensi gradien.</t>
         </is>
       </c>
     </row>
@@ -1643,9 +1774,14 @@
           <t>Adafactor (scale=False, rel=False)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Memfaktorkan momen orde kedua; memangkas memori dari ~4.5GB ke ~50MB.</t>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Adafactor (scale=False, rel=False)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Memfaktorkan momen orde kedua; memangkas memori dari ~2.5GB ke ~35MB.</t>
         </is>
       </c>
     </row>
@@ -1665,9 +1801,14 @@
           <t>2.0e-5 (0.00002)</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>Learning rate standar fine-tuning; 1e-4 terbukti divergen pada DeBERTa.</t>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>2.0e-5 (0.00002)</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Learning rate standar fine-tuning transformer encoder.</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1828,12 @@
           <t>0.01</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Regularisasi L2 standar untuk mencegah overfitting pada dataset kecil.</t>
         </is>
@@ -1709,7 +1855,12 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Menghindari lonjakan memori aktivasi token pada GPU 8GB.</t>
         </is>
@@ -1731,7 +1882,12 @@
           <t>8 langkah</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>8 langkah</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Akumulasi gradien menghasilkan Effective Batch Size = 8.</t>
         </is>
@@ -1753,7 +1909,12 @@
           <t>8 dokumen</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>8 dokumen</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Ukuran batch efektif yang stabil untuk optimasi gradien.</t>
         </is>
@@ -1775,9 +1936,14 @@
           <t>10 Epoch</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>10 epoch per fold; total 80-100 langkah pembaruan bobot per fold.</t>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>10 Epoch</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>10 epoch per fold; total 70-100 langkah pembaruan bobot per fold.</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1955,22 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
+          <t>70 - 100 Langkah</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
           <t>80 - 100 Langkah</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>80 - 100 Langkah</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>80 langkah untuk 51 train doc, 100 langkah untuk 69 train doc.</t>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Langkah optimasi per fold sesuai pembagian fold data latih.</t>
         </is>
       </c>
     </row>
@@ -1819,9 +1990,14 @@
           <t>torch.float32 (model.float())</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>KRITIKAL: DeBERTa di-cast ke FP32 untuk mencegah overflow FP16 pada Adam/Ada.</t>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>torch.float32 (model.float())</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Stabilitas master weight FP32.</t>
         </is>
       </c>
     </row>
@@ -1841,9 +2017,14 @@
           <t>bfloat16 (autocast GPU)</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Didukung native oleh arsitektur RTX 5050; dynamic range sama dengan FP32.</t>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>bfloat16 (autocast GPU)</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Didukung native oleh arsitektur RTX 5050; dynamic range FP32.</t>
         </is>
       </c>
     </row>
@@ -1863,7 +2044,12 @@
           <t>Aktif (gradient_checkpointing_enable)</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Aktif (gradient_checkpointing_enable)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Menukar sedikit komputasi dengan penghematan VRAM aktivasi ~60%.</t>
         </is>
@@ -1885,7 +2071,12 @@
           <t>512 Token</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>512 Token</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Batas panjang konteks maksimum standar model encoder.</t>
         </is>
@@ -1907,7 +2098,12 @@
           <t>64 Token</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>64 Token</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Overlap jendela sliding agar token di batas 512 tidak terpotong.</t>
         </is>
@@ -1929,7 +2125,12 @@
           <t>SEED = 42 + fold_index</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>SEED = 42 + fold_index</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Deterministik penuh untuk reproduksibilitas hasil eksperimen.</t>
         </is>
@@ -1943,15 +2144,20 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
+          <t>96.0% Recall (24/25 token)</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
           <t>100.0% Recall (25/25 token)</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>100.0% Recall (25/25 token)</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Verifikasi bahwa model mampu menghafal label non-O sebelum pelatihan OOF.</t>
         </is>
@@ -1965,15 +2171,20 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
+          <t>700.1 detik (~11.7 menit)</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
           <t>734 detik (~12.2 menit)</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>794 detik (~13.2 menit)</t>
         </is>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Kecepatan eksekusi rata-rata 1.4 - 1.8 detik per langkah optimizer.</t>
         </is>
@@ -1987,17 +2198,22 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
+          <t>4.65 GB / 8.15 GB</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
           <t>4.08 GB / 8.15 GB</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>7.09 GB / 8.15 GB</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Kedua model berhasil dilatih pada workstation RTX 5050 tanpa error OOM.</t>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Ketiga model berhasil dilatih pada workstation RTX 5050 tanpa error OOM.</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2278,7 +2494,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="39" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -2870,100 +3086,415 @@
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>3. Validasi Statistik Bootstrap 1000x Resampling (Exact Macro)</t>
+          <t>3. Evaluasi Per-Fold: treamyracle/indobert-ner-gold (334M) — BEST ENCODER</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Fold</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Train Docs</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Val Docs</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Durasi (s)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Nama Kegiatan</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Nomor</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Penyelenggara</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Tgl Mulai</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Tgl Selesai</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>MACRO Exact</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>MACRO Fuzzy</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D23" s="32" t="n">
+        <v>114</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>0.4348</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0.5294</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>0.3043</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>0.4737</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>0.4737</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>0.4356</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>0.5545</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>0.5238</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>0.3571</v>
+      </c>
+      <c r="J24" s="13" t="n">
+        <v>0.4643</v>
+      </c>
+      <c r="K24" s="13" t="n">
+        <v>0.5714</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D25" s="32" t="n">
+        <v>134.2</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>0.4167</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>0.3438</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>0.5155999999999999</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" s="33" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H26" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I26" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J26" s="13" t="n">
+        <v>0.5405</v>
+      </c>
+      <c r="K26" s="13" t="n">
+        <v>0.6757</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="32" t="n">
+        <v>161.2</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>0.5417</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>Rata-rata OOF</t>
+        </is>
+      </c>
+      <c r="B28" s="35">
+        <f>SUM(B23:B27)/5</f>
+        <v/>
+      </c>
+      <c r="C28" s="35">
+        <f>SUM(C23:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="36">
+        <f>SUM(D23:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>AVERAGE(E23:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>AVERAGE(F23:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>AVERAGE(G23:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>AVERAGE(H23:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>AVERAGE(I23:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="21">
+        <f>AVERAGE(J23:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="21">
+        <f>AVERAGE(K23:K27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>4. Validasi Statistik Bootstrap 1000x Resampling (Exact Macro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>Model Evaluasi</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Sampel Dokumen</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Mean Bootstrap</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Batas Bawah (2.5%)</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Batas Atas (97.5%)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Rentang CI 95% (Width)</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Stabilitas Estimasi</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>mDeBERTa-v3-base (86M)</t>
         </is>
       </c>
-      <c r="B23" s="37" t="n">
+      <c r="B32" s="37" t="n">
         <v>74</v>
       </c>
-      <c r="C23" s="38" t="n">
+      <c r="C32" s="38" t="n">
         <v>0.3478</v>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D32" s="38" t="n">
         <v>0.2895</v>
       </c>
-      <c r="E23" s="38" t="n">
+      <c r="E32" s="38" t="n">
         <v>0.4092</v>
       </c>
-      <c r="F23" s="39">
-        <f>E23-D23</f>
-        <v/>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="F32" s="39">
+        <f>E32-D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>Sangat Stabil (Normal Distribution)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>XLM-RoBERTa-large (560M)</t>
         </is>
       </c>
-      <c r="B24" s="40" t="n">
+      <c r="B33" s="40" t="n">
         <v>74</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C33" s="41" t="n">
         <v>0.4357</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D33" s="41" t="n">
         <v>0.3717</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="E33" s="41" t="n">
         <v>0.5</v>
       </c>
-      <c r="F24" s="42">
-        <f>E24-D24</f>
-        <v/>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="F33" s="42">
+        <f>E33-D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Sangat Stabil (Normal Distribution)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>IndoBERT-ner-gold (334M)</t>
+        </is>
+      </c>
+      <c r="B34" s="37" t="n">
+        <v>74</v>
+      </c>
+      <c r="C34" s="38" t="n">
+        <v>0.4457</v>
+      </c>
+      <c r="D34" s="38" t="n">
+        <v>0.3859</v>
+      </c>
+      <c r="E34" s="38" t="n">
+        <v>0.5082</v>
+      </c>
+      <c r="F34" s="39">
+        <f>E34-D34</f>
+        <v/>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>ENCODER TERBAIK (95% CI Tertinggi: 38.6% - 50.8%)</t>
         </is>
       </c>
     </row>
@@ -2981,18 +3512,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3023,35 +3556,45 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Akurasi IndoBERT</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Penurunan IndoBERT</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Akurasi mDeBERTa</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Penurunan mDeBERTa</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Akurasi XLM-RoBERTa</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Penurunan XLM-RoBERTa</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Akurasi Composite v4.x</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Penurunan Composite v4.x</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Toleransi &amp; Karakteristik</t>
         </is>
@@ -3063,31 +3606,38 @@
           <t>Clean Baseline (Tanpa Noise)</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="40" t="n">
         <v>236</v>
       </c>
-      <c r="C5" s="38" t="n">
-        <v>0.3771</v>
+      <c r="C5" s="41" t="n">
+        <v>0.4703</v>
       </c>
       <c r="D5" s="43">
         <f>C5-C$5</f>
         <v/>
       </c>
-      <c r="E5" s="38" t="n">
-        <v>0.4534</v>
+      <c r="E5" s="41" t="n">
+        <v>0.3771</v>
       </c>
       <c r="F5" s="43">
         <f>E5-E$5</f>
         <v/>
       </c>
-      <c r="G5" s="38" t="n">
-        <v>0.88</v>
+      <c r="G5" s="41" t="n">
+        <v>0.4534</v>
       </c>
       <c r="H5" s="43">
         <f>G5-G$5</f>
         <v/>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="41" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J5" s="43">
+        <f>I5-I$5</f>
+        <v/>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Kondisi teks masukan OCR standar</t>
         </is>
@@ -3099,31 +3649,38 @@
           <t>Mutasi Entitas (UNAIR-&gt;UNS dll)</t>
         </is>
       </c>
-      <c r="B6" s="40" t="n">
+      <c r="B6" s="37" t="n">
         <v>236</v>
       </c>
-      <c r="C6" s="41" t="n">
-        <v>0.3051</v>
+      <c r="C6" s="38" t="n">
+        <v>0.3983</v>
       </c>
       <c r="D6" s="44">
         <f>C6-C$5</f>
         <v/>
       </c>
-      <c r="E6" s="41" t="n">
-        <v>0.3771</v>
+      <c r="E6" s="38" t="n">
+        <v>0.3051</v>
       </c>
       <c r="F6" s="44">
         <f>E6-E$5</f>
         <v/>
       </c>
-      <c r="G6" s="41" t="n">
-        <v>0.806</v>
+      <c r="G6" s="38" t="n">
+        <v>0.3771</v>
       </c>
       <c r="H6" s="44">
         <f>G6-G$5</f>
         <v/>
       </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="I6" s="38" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="J6" s="44">
+        <f>I6-I$5</f>
+        <v/>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>Mengganti nama univ/fakultas/hima ke institusi lain</t>
         </is>
@@ -3135,31 +3692,38 @@
           <t>Perturbasi Noise OCR 10%</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="40" t="n">
         <v>236</v>
       </c>
-      <c r="C7" s="38" t="n">
-        <v>0.25</v>
+      <c r="C7" s="41" t="n">
+        <v>0.3051</v>
       </c>
       <c r="D7" s="43">
         <f>C7-C$5</f>
         <v/>
       </c>
-      <c r="E7" s="38" t="n">
-        <v>0.2924</v>
+      <c r="E7" s="41" t="n">
+        <v>0.25</v>
       </c>
       <c r="F7" s="43">
         <f>E7-E$5</f>
         <v/>
       </c>
-      <c r="G7" s="38" t="n">
-        <v>0.799</v>
+      <c r="G7" s="41" t="n">
+        <v>0.2924</v>
       </c>
       <c r="H7" s="43">
         <f>G7-G$5</f>
         <v/>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="41" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="J7" s="43">
+        <f>I7-I$5</f>
+        <v/>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Simulasi kebingungan karakter 5&lt;-&gt;S, 8&lt;-&gt;B, 0&lt;-&gt;O, 1&lt;-&gt;I</t>
         </is>
@@ -3171,31 +3735,38 @@
           <t>Perturbasi Noise OCR 25%</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n">
+      <c r="B8" s="37" t="n">
         <v>236</v>
       </c>
-      <c r="C8" s="41" t="n">
-        <v>0.2034</v>
+      <c r="C8" s="38" t="n">
+        <v>0.1822</v>
       </c>
       <c r="D8" s="44">
         <f>C8-C$5</f>
         <v/>
       </c>
-      <c r="E8" s="41" t="n">
-        <v>0.1949</v>
+      <c r="E8" s="38" t="n">
+        <v>0.2034</v>
       </c>
       <c r="F8" s="44">
         <f>E8-E$5</f>
         <v/>
       </c>
-      <c r="G8" s="41" t="n">
-        <v>0.698</v>
+      <c r="G8" s="38" t="n">
+        <v>0.1949</v>
       </c>
       <c r="H8" s="44">
         <f>G8-G$5</f>
         <v/>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I8" s="38" t="n">
+        <v>0.698</v>
+      </c>
+      <c r="J8" s="44">
+        <f>I8-I$5</f>
+        <v/>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Tingkat noise OCR sedang pada dokumen buram</t>
         </is>
@@ -3207,31 +3778,38 @@
           <t>Perturbasi Noise OCR 50%</t>
         </is>
       </c>
-      <c r="B9" s="37" t="n">
+      <c r="B9" s="40" t="n">
         <v>236</v>
       </c>
-      <c r="C9" s="38" t="n">
-        <v>0.1017</v>
+      <c r="C9" s="41" t="n">
+        <v>0.089</v>
       </c>
       <c r="D9" s="43">
         <f>C9-C$5</f>
         <v/>
       </c>
-      <c r="E9" s="38" t="n">
-        <v>0.1229</v>
+      <c r="E9" s="41" t="n">
+        <v>0.1017</v>
       </c>
       <c r="F9" s="43">
         <f>E9-E$5</f>
         <v/>
       </c>
-      <c r="G9" s="38" t="n">
-        <v>0.541</v>
+      <c r="G9" s="41" t="n">
+        <v>0.1229</v>
       </c>
       <c r="H9" s="43">
         <f>G9-G$5</f>
         <v/>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="41" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="J9" s="43">
+        <f>I9-I$5</f>
+        <v/>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Tingkat noise OCR ekstrem pada pindaian sangat rusak</t>
         </is>

</xml_diff>

<commit_message>
feat(ner): benchmark zero-shot GLiNER v2.1 dan GLiNER2.5 pada korpus sertifikat (NER-GLINER-001)
- Implementasi runner benchmark tests/benchmark_gliner.py untuk GLiNER v2.1 Multilingual (urchade) dan GLiNER2.5 Base Boundary (arXiv:2507.18546)
- Evaluasi zero-shot schema-driven extraction pada 74 korpus teks Tesseract OCR vs GT v9 + Matcher v2
- GLiNER v2.1 meraih 35.48% framework exact (kebal mutasi OOD dengan drop 0.00pt, latensi 0.077s/c)
- GLiNER2.5 Base meraih 28.71% framework exact (nama kegiatan exact 31.08% / fuzzy 52.70%, latensi 0.052s/c)
- Catat metrik resmi di docs/experiments_ledger.md, runs_summary.md, dan perbarui workbook Excel komparasi_ner_encoder_dan_pipeline.xlsx
</commit_message>
<xml_diff>
--- a/docs/report/komparasi_ner_encoder_dan_pipeline.xlsx
+++ b/docs/report/komparasi_ner_encoder_dan_pipeline.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -870,39 +870,39 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>mDeBERTa-v3-base (86M)</t>
+          <t>GLiNER2.5 Base (arXiv:2507.18546)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>5-Fold CV Token Classif.</t>
+          <t>Zero-Shot Boundary Extractor</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.3484</v>
+        <v>0.2871</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.5129</v>
+        <v>0.3871</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>[28.95%, 40.92%]</t>
+          <t>[23.64%, 34.39%]</t>
         </is>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.2568</v>
+        <v>0.3108</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.5577</v>
+        <v>0.0385</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0.2568</v>
+        <v>0.2027</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.3273</v>
+        <v>0.4545</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>0.4182</v>
+        <v>0.4364</v>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
@@ -911,24 +911,24 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>734 detik (~12.2m)</t>
+          <t>3.9 detik (0.052s/c)</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>4.08 GB</t>
+          <t>~1.8 GB</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Eksplorasi (PASS)</t>
+          <t>Zero-Shot Boundary (PASS)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>XLM-RoBERTa-large (560M)</t>
+          <t>mDeBERTa-v3-base (86M)</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -937,30 +937,30 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.4355</v>
+        <v>0.3484</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.5548</v>
+        <v>0.5129</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>[37.17%, 50.00%]</t>
+          <t>[28.95%, 40.92%]</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3514</v>
+        <v>0.2568</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.5962</v>
+        <v>0.5577</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>0.3784</v>
+        <v>0.2568</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>0.4545</v>
+        <v>0.3273</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>0.4545</v>
+        <v>0.4182</v>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
@@ -969,12 +969,12 @@
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>794 detik (~13.2m)</t>
+          <t>734 detik (~12.2m)</t>
         </is>
       </c>
       <c r="M8" s="12" t="inlineStr">
         <is>
-          <t>7.09 GB (Adafactor)</t>
+          <t>4.08 GB</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
@@ -986,39 +986,39 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
+          <t>GLiNER v2.1 Multilingual (urchade)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>5-Fold CV Token Classif.</t>
+          <t>Zero-Shot Span Bi-Encoder</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.4452</v>
+        <v>0.3548</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.571</v>
+        <v>0.4645</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>[38.59%, 50.82%]</t>
+          <t>[30.10%, 41.31%]</t>
         </is>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.4324</v>
+        <v>0.1622</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.5769</v>
+        <v>0.1346</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>0.3649</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.4909</v>
+        <v>0.5818</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>0.4</v>
+        <v>0.5818</v>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
@@ -1027,318 +1027,378 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>700.1 detik (~11.7m)</t>
+          <t>5.7 detik (0.077s/c)</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>4.65 GB</t>
+          <t>~2.4 GB</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>BEST ENCODER (PASS)</t>
+          <t>Zero-Shot Multi (PASS)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Direct Gemini 3.1 Flash Lite</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Two-Stage Tesseract-to-LLM</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>0.6324</v>
-      </c>
-      <c r="D10" s="16" t="n">
-        <v>0.7378</v>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>[58.78%, 68.92%]</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>0.6216</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>0.5946</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>0.5946</v>
-      </c>
-      <c r="I10" s="18" t="n">
-        <v>0.6757</v>
-      </c>
-      <c r="J10" s="18" t="n">
-        <v>0.6757</v>
-      </c>
-      <c r="K10" s="18" t="n">
-        <v>0.6622</v>
-      </c>
-      <c r="L10" s="17" t="inlineStr">
-        <is>
-          <t>100.6 detik (1.36s/c)</t>
-        </is>
-      </c>
-      <c r="M10" s="17" t="inlineStr">
-        <is>
-          <t>Rp703 (~Rp9.50/c)</t>
-        </is>
-      </c>
-      <c r="N10" s="15" t="inlineStr">
-        <is>
-          <t>PRODUKSI AKTIF (Opt A)</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>XLM-RoBERTa-large (560M)</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>5-Fold CV Token Classif.</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0.4355</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0.5548</v>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>[37.17%, 50.00%]</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>0.3514</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>0.5962</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>0.3784</v>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>0.4545</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>0.4545</v>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>794 detik (~13.2m)</t>
+        </is>
+      </c>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>7.09 GB (Adafactor)</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Eksplorasi (PASS)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>5-Fold CV Token Classif.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.4452</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>[38.59%, 50.82%]</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.4324</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.5769</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.3649</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0.4909</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>700.1 detik (~11.7m)</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>4.65 GB</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>BEST ENCODER (PASS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Direct Gemini 3.1 Flash Lite</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Two-Stage Tesseract-to-LLM</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>0.6324</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>0.7378</v>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>[58.78%, 68.92%]</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>0.6216</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <v>0.5946</v>
+      </c>
+      <c r="H12" s="18" t="n">
+        <v>0.5946</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>0.6757</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>0.6757</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>0.6622</v>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>100.6 detik (1.36s/c)</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>Rp703 (~Rp9.50/c)</t>
+        </is>
+      </c>
+      <c r="N12" s="15" t="inlineStr">
+        <is>
+          <t>PRODUKSI AKTIF (Opt A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Composite v4.x (Pure OCR)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Pure 100% Tesseract OCR + Rules</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>0.771</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D13" s="6" t="n">
         <v>0.8516</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>[72.10%, 81.80%]</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F13" s="8" t="n">
         <v>0.76</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G13" s="8" t="n">
         <v>0.8947000000000001</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H13" s="8" t="n">
         <v>0.36</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I13" s="8" t="n">
         <v>0.9</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J13" s="8" t="n">
         <v>0.9</v>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="K13" s="8" t="n">
         <v>0.6847</v>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>0 detik (Offline)</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>0 GB (CPU Local)</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>Baseline Pure OCR</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Combined v4.2 (Hybrid)</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Hybrid Layer + 3 Pillars &amp; Crop</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C14" s="11" t="n">
         <v>0.8742</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D14" s="11" t="n">
         <v>0.9</v>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>[83.50%, 91.20%]</t>
         </is>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F14" s="13" t="n">
         <v>0.797</v>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="G14" s="13" t="n">
         <v>0.923</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="H14" s="13" t="n">
         <v>0.662</v>
       </c>
-      <c r="I12" s="13" t="n">
+      <c r="I14" s="13" t="n">
         <v>0.909</v>
       </c>
-      <c r="J12" s="13" t="n">
+      <c r="J14" s="13" t="n">
         <v>0.909</v>
       </c>
-      <c r="K12" s="13" t="n">
+      <c r="K14" s="13" t="n">
         <v>0.7682</v>
       </c>
-      <c r="L12" s="12" t="inlineStr">
+      <c r="L14" s="12" t="inlineStr">
         <is>
           <t>0 detik (Offline)</t>
         </is>
       </c>
-      <c r="M12" s="12" t="inlineStr">
+      <c r="M14" s="12" t="inlineStr">
         <is>
           <t>0 GB (CPU Local)</t>
         </is>
       </c>
-      <c r="N12" s="10" t="inlineStr">
+      <c r="N14" s="10" t="inlineStr">
         <is>
           <t>Fallback Produksi</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Rata-rata Model Teruji</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Rata-rata Metrik</t>
         </is>
       </c>
-      <c r="C13" s="21">
-        <f>AVERAGE(C5:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="21">
-        <f>AVERAGE(D5:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="22" t="inlineStr"/>
-      <c r="F13" s="22" t="inlineStr"/>
-      <c r="G13" s="22" t="inlineStr"/>
-      <c r="H13" s="22" t="inlineStr"/>
-      <c r="I13" s="22" t="inlineStr"/>
-      <c r="J13" s="22" t="inlineStr"/>
-      <c r="K13" s="22" t="inlineStr"/>
-      <c r="L13" s="22" t="inlineStr"/>
-      <c r="M13" s="22" t="inlineStr"/>
-      <c r="N13" s="22" t="inlineStr"/>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="C15" s="21">
+        <f>AVERAGE(C5:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="21">
+        <f>AVERAGE(D5:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="22" t="inlineStr"/>
+      <c r="F15" s="22" t="inlineStr"/>
+      <c r="G15" s="22" t="inlineStr"/>
+      <c r="H15" s="22" t="inlineStr"/>
+      <c r="I15" s="22" t="inlineStr"/>
+      <c r="J15" s="22" t="inlineStr"/>
+      <c r="K15" s="22" t="inlineStr"/>
+      <c r="L15" s="22" t="inlineStr"/>
+      <c r="M15" s="22" t="inlineStr"/>
+      <c r="N15" s="22" t="inlineStr"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>ANALISIS DELTA PERFORMANSI VS BASELINE PRE-TRAINED NER V1 (INDOBERT)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Model Komparasi</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Baseline Exact</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Model Exact</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Peningkatan Mutlak (pp)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Peningkatan Relatif (%)</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Kesimpulan Arsitektural</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>IndoBERT Fine-Tuned Gagal (Phase v2)</t>
-        </is>
-      </c>
-      <c r="B17" s="8">
-        <f>C5</f>
-        <v/>
-      </c>
-      <c r="C17" s="8">
-        <f>C6</f>
-        <v/>
-      </c>
-      <c r="D17" s="24">
-        <f>C17-B17</f>
-        <v/>
-      </c>
-      <c r="E17" s="25">
-        <f>(C17-B17)/B17</f>
-        <v/>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Anjlok -11.3pp akibat catastrophic forgetting pada 59 sampel dan ketiadaan weighted loss.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>mDeBERTa-v3-base (86M)</t>
-        </is>
-      </c>
-      <c r="B18" s="13">
-        <f>C5</f>
-        <v/>
-      </c>
-      <c r="C18" s="13">
-        <f>C7</f>
-        <v/>
-      </c>
-      <c r="D18" s="26">
-        <f>C18-B18</f>
-        <v/>
-      </c>
-      <c r="E18" s="27">
-        <f>(C18-B18)/B18</f>
-        <v/>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Peningkatan substansial (+22.04pp) pada recall entitas non-O via FP32 &amp; soft-capping.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>XLM-RoBERTa-large (560M)</t>
+          <t>IndoBERT Fine-Tuned Gagal (Phase v2)</t>
         </is>
       </c>
       <c r="B19" s="8">
@@ -1346,7 +1406,7 @@
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>C8</f>
+        <f>C6</f>
         <v/>
       </c>
       <c r="D19" s="24">
@@ -1359,14 +1419,14 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Model 560M melompat +30.75pp; representasi BPE multilingual sangat kuat.</t>
+          <t>Anjlok -11.3pp akibat catastrophic forgetting pada 59 sampel dan ketiadaan weighted loss.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
+          <t>GLiNER2.5 Base (arXiv:2507.18546)</t>
         </is>
       </c>
       <c r="B20" s="13">
@@ -1374,7 +1434,7 @@
         <v/>
       </c>
       <c r="C20" s="13">
-        <f>C9</f>
+        <f>C7</f>
         <v/>
       </c>
       <c r="D20" s="26">
@@ -1387,14 +1447,14 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>ENCODER TERBAIK (+31.72pp vs pre-trained, +0.97pp vs XLM-RoBERTa-large, kegiatan melonjak ke 43.2%).</t>
+          <t>Zero-shot boundary extractor melompat +15.91pp; nama kegiatan exact mencapai 31.1%.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Direct Gemini 3.1 Flash Lite</t>
+          <t>mDeBERTa-v3-base (86M)</t>
         </is>
       </c>
       <c r="B21" s="8">
@@ -1402,7 +1462,7 @@
         <v/>
       </c>
       <c r="C21" s="8">
-        <f>C10</f>
+        <f>C8</f>
         <v/>
       </c>
       <c r="D21" s="24">
@@ -1415,14 +1475,14 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>LLM murni melampaui seluruh encoder lokal tanpa memerlukan fine-tuning.</t>
+          <t>Peningkatan substansial (+22.04pp) pada recall entitas non-O via FP32 &amp; soft-capping.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Composite v4.x (Pure OCR Rules)</t>
+          <t>GLiNER v2.1 Multilingual (urchade)</t>
         </is>
       </c>
       <c r="B22" s="13">
@@ -1430,7 +1490,7 @@
         <v/>
       </c>
       <c r="C22" s="13">
-        <f>C11</f>
+        <f>C9</f>
         <v/>
       </c>
       <c r="D22" s="26">
@@ -1443,14 +1503,14 @@
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Rule deterministik offline tetap paling unggul pada domain penanggalan &amp; nomor.</t>
+          <t>Zero-shot multilingual melompat +22.68pp; tanggal 58.2% &amp; mutasi OOD drop 0.0pt.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Combined v4.2 (Hybrid Pipeline)</t>
+          <t>XLM-RoBERTa-large (560M)</t>
         </is>
       </c>
       <c r="B23" s="8">
@@ -1458,7 +1518,7 @@
         <v/>
       </c>
       <c r="C23" s="8">
-        <f>C12</f>
+        <f>C10</f>
         <v/>
       </c>
       <c r="D23" s="24">
@@ -1470,6 +1530,118 @@
         <v/>
       </c>
       <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Model 560M melompat +30.75pp; representasi BPE multilingual sangat kuat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>IndoBERT-ner-gold Fine-Tuned (334M)</t>
+        </is>
+      </c>
+      <c r="B24" s="13">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C24" s="13">
+        <f>C11</f>
+        <v/>
+      </c>
+      <c r="D24" s="26">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+      <c r="E24" s="27">
+        <f>(C24-B24)/B24</f>
+        <v/>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>ENCODER TERBAIK (+31.72pp vs pre-trained, +0.97pp vs XLM-RoBERTa-large, kegiatan 43.2%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Direct Gemini 3.1 Flash Lite</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C25" s="8">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="D25" s="24">
+        <f>C25-B25</f>
+        <v/>
+      </c>
+      <c r="E25" s="25">
+        <f>(C25-B25)/B25</f>
+        <v/>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>LLM murni melampaui seluruh encoder lokal tanpa memerlukan fine-tuning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Composite v4.x (Pure OCR Rules)</t>
+        </is>
+      </c>
+      <c r="B26" s="13">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C26" s="13">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="D26" s="26">
+        <f>C26-B26</f>
+        <v/>
+      </c>
+      <c r="E26" s="27">
+        <f>(C26-B26)/B26</f>
+        <v/>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Rule deterministik offline tetap paling unggul pada domain penanggalan &amp; nomor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Combined v4.2 (Hybrid Pipeline)</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="C27" s="8">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="D27" s="24">
+        <f>C27-B27</f>
+        <v/>
+      </c>
+      <c r="E27" s="25">
+        <f>(C27-B27)/B27</f>
+        <v/>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Pipeline komposit offline terbaik, unggul +74.62pp dibanding baseline NER v1.</t>
         </is>
@@ -3512,20 +3684,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3556,47 +3732,67 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Akurasi GLiNER v2.1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Drop GLiNER v2.1</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Akurasi GLiNER2.5</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Drop GLiNER2.5</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Akurasi IndoBERT</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Penurunan IndoBERT</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Drop IndoBERT</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Akurasi mDeBERTa</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Penurunan mDeBERTa</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Drop mDeBERTa</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Akurasi XLM-RoBERTa</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Penurunan XLM-RoBERTa</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Drop XLM-RoBERTa</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Akurasi Composite v4.x</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Penurunan Composite v4.x</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Toleransi &amp; Karakteristik</t>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Drop Composite v4.x</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Toleransi &amp; Karakteristik Arsitektural</t>
         </is>
       </c>
     </row>
@@ -3610,34 +3806,48 @@
         <v>236</v>
       </c>
       <c r="C5" s="41" t="n">
-        <v>0.4703</v>
+        <v>0.3517</v>
       </c>
       <c r="D5" s="43">
         <f>C5-C$5</f>
         <v/>
       </c>
       <c r="E5" s="41" t="n">
-        <v>0.3771</v>
+        <v>0.2839</v>
       </c>
       <c r="F5" s="43">
         <f>E5-E$5</f>
         <v/>
       </c>
       <c r="G5" s="41" t="n">
-        <v>0.4534</v>
+        <v>0.4703</v>
       </c>
       <c r="H5" s="43">
         <f>G5-G$5</f>
         <v/>
       </c>
       <c r="I5" s="41" t="n">
-        <v>0.88</v>
+        <v>0.3771</v>
       </c>
       <c r="J5" s="43">
         <f>I5-I$5</f>
         <v/>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="41" t="n">
+        <v>0.4534</v>
+      </c>
+      <c r="L5" s="43">
+        <f>K5-K$5</f>
+        <v/>
+      </c>
+      <c r="M5" s="41" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="N5" s="43">
+        <f>M5-M$5</f>
+        <v/>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Kondisi teks masukan OCR standar</t>
         </is>
@@ -3653,36 +3863,50 @@
         <v>236</v>
       </c>
       <c r="C6" s="38" t="n">
-        <v>0.3983</v>
+        <v>0.3517</v>
       </c>
       <c r="D6" s="44">
         <f>C6-C$5</f>
         <v/>
       </c>
       <c r="E6" s="38" t="n">
-        <v>0.3051</v>
+        <v>0.2797</v>
       </c>
       <c r="F6" s="44">
         <f>E6-E$5</f>
         <v/>
       </c>
       <c r="G6" s="38" t="n">
-        <v>0.3771</v>
+        <v>0.3983</v>
       </c>
       <c r="H6" s="44">
         <f>G6-G$5</f>
         <v/>
       </c>
       <c r="I6" s="38" t="n">
-        <v>0.806</v>
+        <v>0.3051</v>
       </c>
       <c r="J6" s="44">
         <f>I6-I$5</f>
         <v/>
       </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>Mengganti nama univ/fakultas/hima ke institusi lain</t>
+      <c r="K6" s="38" t="n">
+        <v>0.3771</v>
+      </c>
+      <c r="L6" s="44">
+        <f>K6-K$5</f>
+        <v/>
+      </c>
+      <c r="M6" s="38" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="N6" s="44">
+        <f>M6-M$5</f>
+        <v/>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>GLiNER kebal mutasi (drop 0.0pt) karena berbasis query skema dinamis</t>
         </is>
       </c>
     </row>
@@ -3696,34 +3920,48 @@
         <v>236</v>
       </c>
       <c r="C7" s="41" t="n">
-        <v>0.3051</v>
+        <v>0.2712</v>
       </c>
       <c r="D7" s="43">
         <f>C7-C$5</f>
         <v/>
       </c>
       <c r="E7" s="41" t="n">
-        <v>0.25</v>
+        <v>0.2288</v>
       </c>
       <c r="F7" s="43">
         <f>E7-E$5</f>
         <v/>
       </c>
       <c r="G7" s="41" t="n">
-        <v>0.2924</v>
+        <v>0.3051</v>
       </c>
       <c r="H7" s="43">
         <f>G7-G$5</f>
         <v/>
       </c>
       <c r="I7" s="41" t="n">
-        <v>0.799</v>
+        <v>0.25</v>
       </c>
       <c r="J7" s="43">
         <f>I7-I$5</f>
         <v/>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="41" t="n">
+        <v>0.2924</v>
+      </c>
+      <c r="L7" s="43">
+        <f>K7-K$5</f>
+        <v/>
+      </c>
+      <c r="M7" s="41" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="N7" s="43">
+        <f>M7-M$5</f>
+        <v/>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>Simulasi kebingungan karakter 5&lt;-&gt;S, 8&lt;-&gt;B, 0&lt;-&gt;O, 1&lt;-&gt;I</t>
         </is>
@@ -3739,34 +3977,48 @@
         <v>236</v>
       </c>
       <c r="C8" s="38" t="n">
-        <v>0.1822</v>
+        <v>0.178</v>
       </c>
       <c r="D8" s="44">
         <f>C8-C$5</f>
         <v/>
       </c>
       <c r="E8" s="38" t="n">
-        <v>0.2034</v>
+        <v>0.1525</v>
       </c>
       <c r="F8" s="44">
         <f>E8-E$5</f>
         <v/>
       </c>
       <c r="G8" s="38" t="n">
-        <v>0.1949</v>
+        <v>0.1822</v>
       </c>
       <c r="H8" s="44">
         <f>G8-G$5</f>
         <v/>
       </c>
       <c r="I8" s="38" t="n">
-        <v>0.698</v>
+        <v>0.2034</v>
       </c>
       <c r="J8" s="44">
         <f>I8-I$5</f>
         <v/>
       </c>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="K8" s="38" t="n">
+        <v>0.1949</v>
+      </c>
+      <c r="L8" s="44">
+        <f>K8-K$5</f>
+        <v/>
+      </c>
+      <c r="M8" s="38" t="n">
+        <v>0.698</v>
+      </c>
+      <c r="N8" s="44">
+        <f>M8-M$5</f>
+        <v/>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
         <is>
           <t>Tingkat noise OCR sedang pada dokumen buram</t>
         </is>
@@ -3782,34 +4034,48 @@
         <v>236</v>
       </c>
       <c r="C9" s="41" t="n">
-        <v>0.089</v>
+        <v>0.1017</v>
       </c>
       <c r="D9" s="43">
         <f>C9-C$5</f>
         <v/>
       </c>
       <c r="E9" s="41" t="n">
-        <v>0.1017</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="F9" s="43">
         <f>E9-E$5</f>
         <v/>
       </c>
       <c r="G9" s="41" t="n">
-        <v>0.1229</v>
+        <v>0.089</v>
       </c>
       <c r="H9" s="43">
         <f>G9-G$5</f>
         <v/>
       </c>
       <c r="I9" s="41" t="n">
-        <v>0.541</v>
+        <v>0.1017</v>
       </c>
       <c r="J9" s="43">
         <f>I9-I$5</f>
         <v/>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="41" t="n">
+        <v>0.1229</v>
+      </c>
+      <c r="L9" s="43">
+        <f>K9-K$5</f>
+        <v/>
+      </c>
+      <c r="M9" s="41" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="N9" s="43">
+        <f>M9-M$5</f>
+        <v/>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Tingkat noise OCR ekstrem pada pindaian sangat rusak</t>
         </is>

</xml_diff>